<commit_message>
including edit user function
</commit_message>
<xml_diff>
--- a/clients.xlsx
+++ b/clients.xlsx
@@ -1068,7 +1068,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>athmania</t>
+          <t>algeria</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1078,7 +1078,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>athmania</t>
+          <t>algeria</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
adding edit user, search user, all work fine
</commit_message>
<xml_diff>
--- a/clients.xlsx
+++ b/clients.xlsx
@@ -1084,32 +1084,80 @@
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>2023</v>
-      </c>
-      <c r="B25" t="inlineStr"/>
-      <c r="C25" t="inlineStr"/>
+        <v>2000</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Salamandre</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Salamandre</t>
+        </is>
+      </c>
       <c r="D25" t="inlineStr"/>
-      <c r="E25" t="inlineStr"/>
-      <c r="F25" t="inlineStr"/>
-      <c r="G25" t="inlineStr"/>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Alger</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>mezouani.nadjib@gmail.com</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Salamandre</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>2024</v>
-      </c>
-      <c r="B26" t="inlineStr"/>
-      <c r="C26" t="inlineStr"/>
+        <v>2000</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
       <c r="D26" t="inlineStr"/>
-      <c r="E26" t="inlineStr"/>
-      <c r="F26" t="inlineStr"/>
-      <c r="G26" t="inlineStr"/>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>tes</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>tes@tas.com</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>2025</v>
-      </c>
-      <c r="B27" t="inlineStr"/>
-      <c r="C27" t="inlineStr"/>
+        <v>2000</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>papa</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>papa</t>
+        </is>
+      </c>
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr"/>
       <c r="F27" t="inlineStr"/>
@@ -1117,21 +1165,53 @@
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>2026</v>
-      </c>
-      <c r="B28" t="inlineStr"/>
-      <c r="C28" t="inlineStr"/>
-      <c r="D28" t="inlineStr"/>
-      <c r="E28" t="inlineStr"/>
-      <c r="F28" t="inlineStr"/>
-      <c r="G28" t="inlineStr"/>
+        <v>2000</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>mama</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>mama</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>423403409</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>ama</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>kama</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>mam</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>2027</v>
-      </c>
-      <c r="B29" t="inlineStr"/>
-      <c r="C29" t="inlineStr"/>
+        <v>2000</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>lana</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>lana</t>
+        </is>
+      </c>
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr"/>
       <c r="F29" t="inlineStr"/>
@@ -1139,32 +1219,80 @@
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>2028</v>
-      </c>
-      <c r="B30" t="inlineStr"/>
-      <c r="C30" t="inlineStr"/>
-      <c r="D30" t="inlineStr"/>
-      <c r="E30" t="inlineStr"/>
-      <c r="F30" t="inlineStr"/>
-      <c r="G30" t="inlineStr"/>
+        <v>2000</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Mr Nadjib</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>0555371257</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Alger</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>nadjib44@gmail.com</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Sarl SALAMANDRE</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>2029</v>
-      </c>
-      <c r="B31" t="inlineStr"/>
-      <c r="C31" t="inlineStr"/>
+        <v>2000</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>mourad</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
       <c r="D31" t="inlineStr"/>
-      <c r="E31" t="inlineStr"/>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
       <c r="F31" t="inlineStr"/>
-      <c r="G31" t="inlineStr"/>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>2030</v>
-      </c>
-      <c r="B32" t="inlineStr"/>
-      <c r="C32" t="inlineStr"/>
+        <v>2000</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>pilo</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>loo</t>
+        </is>
+      </c>
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr"/>
       <c r="F32" t="inlineStr"/>

</xml_diff>